<commit_message>
add one new result to RQ1 and RQ2
</commit_message>
<xml_diff>
--- a/experiment/RQ1_landscape.xlsx
+++ b/experiment/RQ1_landscape.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\research\7-MATester\agents\MATester\experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89790340-57CD-4ABE-B92C-9FD3B9A9A4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66D37644-7A36-4B65-A9A3-BDD1D7B275BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -267,10 +267,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>21/21</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>61/68</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -330,6 +326,10 @@
   </si>
   <si>
     <t>percentage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>22/22</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -960,27 +960,27 @@
         <v>55</v>
       </c>
       <c r="B4">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C4">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D4">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B5">
         <f>SUM(B2:B4)</f>
-        <v>1268</v>
+        <v>1272</v>
       </c>
       <c r="C5">
         <f t="shared" ref="C5:D5" si="0">SUM(C2:C4)</f>
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -1019,25 +1019,25 @@
         <v>5</v>
       </c>
       <c r="E1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" t="s">
         <v>61</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>62</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" t="s">
         <v>63</v>
       </c>
-      <c r="H1" t="s">
-        <v>60</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>64</v>
       </c>
-      <c r="J1" t="s">
-        <v>65</v>
-      </c>
       <c r="K1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1045,7 +1045,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1081,7 +1081,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3">
         <v>28</v>
@@ -1117,7 +1117,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1150,11 +1150,11 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5">
-        <f>48+61+21</f>
-        <v>130</v>
+        <f>48+61+22</f>
+        <v>131</v>
       </c>
       <c r="C5">
         <f>SUM(C2:C4)</f>
@@ -1294,7 +1294,7 @@
         <v>55</v>
       </c>
       <c r="B4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1313,16 +1313,16 @@
       </c>
       <c r="H4">
         <f>SUM(B4:G4)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5">
         <f>SUM(B2:B4)</f>
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C5">
         <f t="shared" ref="C5:H5" si="0">SUM(C2:C4)</f>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -1388,7 +1388,7 @@
         <v>45</v>
       </c>
       <c r="I1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -1448,7 +1448,7 @@
         <v>55</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1471,11 +1471,11 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5">
         <f>SUM(B2:B4)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5">
         <f t="shared" ref="C5:G5" si="0">SUM(C2:C4)</f>
@@ -1504,11 +1504,11 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6">
         <f>B5/I5</f>
-        <v>0.38235294117647056</v>
+        <v>0.41176470588235292</v>
       </c>
       <c r="C6">
         <f>C5/I5</f>
@@ -1634,7 +1634,7 @@
         <v>33</v>
       </c>
       <c r="S2" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="T2" s="11" t="s">
         <v>35</v>
@@ -1933,7 +1933,7 @@
         <v>0</v>
       </c>
       <c r="R6" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6" s="8">
         <v>0</v>
@@ -1955,12 +1955,12 @@
       </c>
       <c r="Y6" s="8">
         <f>SUM(B6:X6)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7">
         <f>SUM(B4:B6)</f>
@@ -2028,7 +2028,7 @@
       </c>
       <c r="R7">
         <f t="shared" ref="R7" si="10">SUM(R4:R6)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S7">
         <f t="shared" ref="S7" si="11">SUM(S4:S6)</f>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="I8">
         <f>SUM(I7:S7)</f>
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="T8">
         <f>SUM(T7:X7)</f>
@@ -2186,13 +2186,13 @@
         <v>33</v>
       </c>
       <c r="S2" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="T2" s="23" t="s">
         <v>35</v>
       </c>
       <c r="U2" s="31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="V2" s="32"/>
       <c r="W2" s="12" t="s">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="Y3" s="27"/>
       <c r="Z3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
@@ -2494,7 +2494,7 @@
         <v>0</v>
       </c>
       <c r="R6" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6" s="8">
         <v>0</v>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="Y6" s="8">
         <f>SUM(B6:X6)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Z6">
         <v>9</v>
@@ -2524,7 +2524,7 @@
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7">
         <f>SUM(B4:B6)</f>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="R7">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S7">
         <f t="shared" si="0"/>
@@ -2625,7 +2625,7 @@
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B8">
         <f>B7/Z7</f>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="R8">
         <f>R7/Z7</f>
-        <v>0.14705882352941177</v>
+        <v>0.17647058823529413</v>
       </c>
       <c r="S8">
         <f>S7/Z7</f>
@@ -2759,12 +2759,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="U9:V9"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:N9"/>
-    <mergeCell ref="P9:Q9"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="I1:S1"/>
@@ -2776,6 +2770,12 @@
     <mergeCell ref="L2:N2"/>
     <mergeCell ref="P2:Q2"/>
     <mergeCell ref="U2:V2"/>
+    <mergeCell ref="U9:V9"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="P9:Q9"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2908,7 +2908,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="J4">
         <f>SUM(B4:I4)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5">
         <f>SUM(B2:B4)</f>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
@@ -3015,7 +3015,7 @@
         <v>21</v>
       </c>
       <c r="K1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -3104,7 +3104,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="J4">
         <f>SUM(B4:I4)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K4">
         <v>9</v>
@@ -3128,7 +3128,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5">
         <f>SUM(B2:B4)</f>
@@ -3144,7 +3144,7 @@
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
@@ -3169,7 +3169,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6">
         <f>B5/K5</f>
@@ -3185,7 +3185,7 @@
       </c>
       <c r="E6">
         <f>E5/K5</f>
-        <v>0.11764705882352941</v>
+        <v>0.14705882352941177</v>
       </c>
       <c r="F6">
         <f>F5/K5</f>

</xml_diff>